<commit_message>
less error on 27 simulations only in 27/27 since ssp3-7.0 scenario
</commit_message>
<xml_diff>
--- a/e1_2_disclosure_table.xlsx
+++ b/e1_2_disclosure_table.xlsx
@@ -2993,7 +2993,7 @@
         <v>26</v>
       </c>
       <c r="F237">
-        <v>0</v>
+        <v>0.009686979362018353</v>
       </c>
       <c r="G237">
         <v>0.009805714028351783</v>
@@ -6863,7 +6863,7 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>0.08254106257287852</v>
+        <v>0.09222804193489686</v>
       </c>
       <c r="C2">
         <v>0.01228151887003103</v>
@@ -6964,13 +6964,13 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <v>0.002275709406225884</v>
+        <v>0.01196268876824424</v>
       </c>
       <c r="E2">
-        <v>0.0009999999776482583</v>
+        <v>0.009686979362018353</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6">

</xml_diff>